<commit_message>
page-log: add 1 new page(s) from nightly 2026-06-26
</commit_message>
<xml_diff>
--- a/trackers/all-sites.xlsx
+++ b/trackers/all-sites.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,8 +59,13 @@
       <color rgb="00888888"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000000CC"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -80,6 +85,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD700"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -141,10 +151,22 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -623,17 +645,17 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>nausea-vomiting-chemotherapy</t>
+          <t>what-is-a-chemo-port</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>https://cioncancerdrowais.com/nausea-vomiting-chemotherapy.html</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
+          <t>https://cioncancerdrowais.com/what-is-a-chemo-port.html</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Published ✓</t>
         </is>
       </c>
     </row>
@@ -658,7 +680,7 @@
           <t>https://cioncancerdrowais.com/hair-loss-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -685,7 +707,7 @@
           <t>https://cioncancerdrowais.com/cancer-fatigue-management.html</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -712,7 +734,7 @@
           <t>https://cioncancerdrowais.com/cancer-nutrition-diet.html</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -739,7 +761,7 @@
           <t>https://cioncancerdrowais.com/breast-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -766,7 +788,7 @@
           <t>https://cioncancerdrowais.com/cervical-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -793,7 +815,7 @@
           <t>https://cioncancerdrowais.com/ovarian-cancer-diagnosis.html</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -820,7 +842,7 @@
           <t>https://cioncancerdrowais.com/colorectal-cancer-screening.html</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -847,7 +869,7 @@
           <t>https://cioncancerdrowais.com/what-is-lymphoma.html</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -874,7 +896,7 @@
           <t>https://cioncancerdrowais.com/types-of-leukemia.html</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -901,7 +923,7 @@
           <t>https://cioncancerdrowais.com/multiple-myeloma-treatment.html</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -928,7 +950,7 @@
           <t>https://cioncancerdrowais.com/blood-tests-cancer-diagnosis.html</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -955,7 +977,7 @@
           <t>https://cioncancerdrowais.com/pet-ct-scan-explained.html</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -982,7 +1004,7 @@
           <t>https://cioncancerdrowais.com/palliative-care-cancer.html</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1009,7 +1031,7 @@
           <t>https://cioncancerdrowais.com/genetic-testing-cancer-risk.html</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1036,7 +1058,7 @@
           <t>https://cioncancerdrowais.com/hereditary-cancer-syndromes.html</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1063,7 +1085,7 @@
           <t>https://cioncancerdrowais.com/managing-cancer-recurrence.html</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1090,7 +1112,7 @@
           <t>https://cioncancerdrowais.com/immunotherapy-side-effects.html</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1117,7 +1139,7 @@
           <t>https://cioncancerdrowais.com/targeted-therapy-explained.html</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1144,7 +1166,7 @@
           <t>https://cioncancerdrowais.com/oral-chemotherapy-medications.html</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1171,7 +1193,7 @@
           <t>https://cioncancerdrowais.com/chemotherapy-port-explained.html</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1198,7 +1220,7 @@
           <t>https://cioncancerdrowais.com/cancer-clinical-trials-india.html</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1225,7 +1247,7 @@
           <t>https://cioncancerdrowais.com/questions-to-ask-oncologist.html</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1252,7 +1274,7 @@
           <t>https://cioncancerdrowais.com/cancer-survivorship-care.html</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1279,7 +1301,7 @@
           <t>https://cioncancerdrowais.com/fertility-preservation-chemotherapy.html</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1306,7 +1328,7 @@
           <t>https://cioncancerdrowais.com/mouth-sores-chemotherapy.html</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1333,7 +1355,7 @@
           <t>https://cioncancerdrowais.com/chemotherapy-neuropathy.html</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1360,7 +1382,7 @@
           <t>https://cioncancerdrowais.com/cancer-diabetes-management.html</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1387,7 +1409,7 @@
           <t>https://cioncancerdrowais.com/blood-transfusion-cancer.html</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1414,7 +1436,7 @@
           <t>https://cioncancerdrowais.com/anti-nausea-medications-chemotherapy.html</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1441,7 +1463,7 @@
           <t>https://cioncancerdrowais.com/cancer-diagnosis-process.html</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1468,7 +1490,7 @@
           <t>https://cioncancerdrowais.com/reading-pathology-report.html</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1495,7 +1517,7 @@
           <t>https://cioncancerdrowais.com/cancer-prognosis-explained.html</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1522,7 +1544,7 @@
           <t>https://cioncancerdrowais.com/cancer-related-anaemia.html</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1549,7 +1571,7 @@
           <t>https://cioncancerdrowais.com/skin-changes-chemotherapy.html</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1576,7 +1598,7 @@
           <t>https://cioncancerdrowais.com/cancer-treatment-pregnancy.html</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1603,7 +1625,7 @@
           <t>https://cioncancerdrowais.com/triple-negative-breast-cancer.html</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1630,7 +1652,7 @@
           <t>https://cioncancerdrowais.com/her2-positive-breast-cancer.html</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1657,7 +1679,7 @@
           <t>https://cioncancerdrowais.com/stomach-cancer-symptoms.html</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1684,7 +1706,7 @@
           <t>https://cioncancerdrowais.com/kidney-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1711,7 +1733,7 @@
           <t>https://cioncancerdrowais.com/bladder-cancer-diagnosis.html</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1738,7 +1760,7 @@
           <t>https://cioncancerdrowais.com/thyroid-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E46" s="12" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1765,7 +1787,7 @@
           <t>https://cioncancerdrowais.com/prostate-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E47" s="11" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1792,7 +1814,7 @@
           <t>https://cioncancerdrowais.com/esophageal-cancer-symptoms.html</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1819,7 +1841,7 @@
           <t>https://cioncancerdrowais.com/cervical-cancer-hpv-vaccine.html</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1846,7 +1868,7 @@
           <t>https://cioncancerdrowais.com/cancer-screening-india.html</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1873,7 +1895,7 @@
           <t>https://cioncancerdrowais.com/why-cancer-second-opinion.html</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1900,7 +1922,7 @@
           <t>https://cioncancerdrowais.com/preparing-for-chemotherapy.html</t>
         </is>
       </c>
-      <c r="E52" s="12" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1927,7 +1949,7 @@
           <t>https://cioncancerdrowais.com/cancer-caregiver-guide.html</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E53" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -1954,7 +1976,7 @@
           <t>https://cioncancerdrowais.com/cancer-pain-relief.html</t>
         </is>
       </c>
-      <c r="E54" s="12" t="inlineStr">
+      <c r="E54" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -2660,29 +2682,29 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Types of cancer surgery</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>types-cancer-surgery</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>https://cioncancerdrvinay.com/types-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Today →</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2729,7 @@
           <t>https://cioncancerdrvinay.com/laparoscopic-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -2734,7 +2756,7 @@
           <t>https://cioncancerdrvinay.com/lumpectomy-breast-surgery.html</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -2761,7 +2783,7 @@
           <t>https://cioncancerdrvinay.com/mastectomy-types-recovery.html</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -2788,7 +2810,7 @@
           <t>https://cioncancerdrvinay.com/sentinel-lymph-node-biopsy.html</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -2815,7 +2837,7 @@
           <t>https://cioncancerdrvinay.com/thyroid-surgery-cancer.html</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -2842,7 +2864,7 @@
           <t>https://cioncancerdrvinay.com/colorectal-surgery.html</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -2869,7 +2891,7 @@
           <t>https://cioncancerdrvinay.com/colostomy-explained.html</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -2896,7 +2918,7 @@
           <t>https://cioncancerdrvinay.com/ileostomy-care.html</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -2923,7 +2945,7 @@
           <t>https://cioncancerdrvinay.com/liver-resection-surgery.html</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -2950,7 +2972,7 @@
           <t>https://cioncancerdrvinay.com/splenectomy-cancer.html</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -2977,7 +2999,7 @@
           <t>https://cioncancerdrvinay.com/nephrectomy-surgery.html</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3004,7 +3026,7 @@
           <t>https://cioncancerdrvinay.com/ovarian-debulking-surgery.html</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3031,7 +3053,7 @@
           <t>https://cioncancerdrvinay.com/cancer-surgery-wound-care.html</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3058,7 +3080,7 @@
           <t>https://cioncancerdrvinay.com/post-surgery-pain-management.html</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3085,7 +3107,7 @@
           <t>https://cioncancerdrvinay.com/cancer-surgery-recovery.html</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3112,7 +3134,7 @@
           <t>https://cioncancerdrvinay.com/cancer-surgery-complications.html</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3139,7 +3161,7 @@
           <t>https://cioncancerdrvinay.com/dvt-prevention-after-surgery.html</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3166,7 +3188,7 @@
           <t>https://cioncancerdrvinay.com/pre-surgery-preparation.html</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3193,7 +3215,7 @@
           <t>https://cioncancerdrvinay.com/nutrition-before-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3220,7 +3242,7 @@
           <t>https://cioncancerdrvinay.com/cancer-surgery-anaesthesia.html</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3247,7 +3269,7 @@
           <t>https://cioncancerdrvinay.com/surgical-staging-cancer.html</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3274,7 +3296,7 @@
           <t>https://cioncancerdrvinay.com/curative-vs-palliative-surgery.html</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3301,7 +3323,7 @@
           <t>https://cioncancerdrvinay.com/breast-reconstruction-after-mastectomy.html</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3328,7 +3350,7 @@
           <t>https://cioncancerdrvinay.com/port-insertion-surgery.html</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3355,7 +3377,7 @@
           <t>https://cioncancerdrvinay.com/vats-thoracoscopy.html</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3382,7 +3404,7 @@
           <t>https://cioncancerdrvinay.com/esophagectomy-surgery.html</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3409,7 +3431,7 @@
           <t>https://cioncancerdrvinay.com/gastrectomy-types.html</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3436,7 +3458,7 @@
           <t>https://cioncancerdrvinay.com/pancreatectomy-procedure.html</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3463,7 +3485,7 @@
           <t>https://cioncancerdrvinay.com/whipple-surgery-recovery.html</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3490,7 +3512,7 @@
           <t>https://cioncancerdrvinay.com/hernia-after-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3517,7 +3539,7 @@
           <t>https://cioncancerdrvinay.com/scar-management-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3544,7 +3566,7 @@
           <t>https://cioncancerdrvinay.com/cancer-surgery-elderly.html</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3571,7 +3593,7 @@
           <t>https://cioncancerdrvinay.com/cancer-surgery-cost-hyderabad.html</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3598,7 +3620,7 @@
           <t>https://cioncancerdrvinay.com/cancer-surgery-questions.html</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3625,7 +3647,7 @@
           <t>https://cioncancerdrvinay.com/life-after-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3652,7 +3674,7 @@
           <t>https://cioncancerdrvinay.com/robotic-cancer-surgery-india.html</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3679,7 +3701,7 @@
           <t>https://cioncancerdrvinay.com/abdominal-cancer-surgery-recovery.html</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3706,7 +3728,7 @@
           <t>https://cioncancerdrvinay.com/rectal-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3733,7 +3755,7 @@
           <t>https://cioncancerdrvinay.com/parathyroid-surgery.html</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3760,7 +3782,7 @@
           <t>https://cioncancerdrvinay.com/adrenalectomy-procedure.html</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3787,7 +3809,7 @@
           <t>https://cioncancerdrvinay.com/pelvic-exenteration-surgery.html</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3814,7 +3836,7 @@
           <t>https://cioncancerdrvinay.com/lymph-node-removal-surgery.html</t>
         </is>
       </c>
-      <c r="E46" s="12" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3841,7 +3863,7 @@
           <t>https://cioncancerdrvinay.com/cancer-biopsy-types.html</t>
         </is>
       </c>
-      <c r="E47" s="11" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3868,7 +3890,7 @@
           <t>https://cioncancerdrvinay.com/intraoperative-frozen-section.html</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3895,7 +3917,7 @@
           <t>https://cioncancerdrvinay.com/cancer-resection-margins.html</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3922,7 +3944,7 @@
           <t>https://cioncancerdrvinay.com/cancer-surgery-second-opinion.html</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3949,7 +3971,7 @@
           <t>https://cioncancerdrvinay.com/day-surgery-cancer.html</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -3976,7 +3998,7 @@
           <t>https://cioncancerdrvinay.com/reconstructive-flap-surgery.html</t>
         </is>
       </c>
-      <c r="E52" s="12" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4003,7 +4025,7 @@
           <t>https://cioncancerdrvinay.com/questions-for-cancer-surgeon.html</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E53" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4680,29 +4702,29 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Melanoma surgery and margins</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>melanoma-surgery</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>https://cioncancerdrmurali.com/melanoma-surgery.html</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Today →</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4749,7 @@
           <t>https://cioncancerdrmurali.com/skin-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4754,7 +4776,7 @@
           <t>https://cioncancerdrmurali.com/retroperitoneal-sarcoma-surgery.html</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4781,7 +4803,7 @@
           <t>https://cioncancerdrmurali.com/leiomyosarcoma-treatment.html</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4808,7 +4830,7 @@
           <t>https://cioncancerdrmurali.com/liposarcoma-surgery.html</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4835,7 +4857,7 @@
           <t>https://cioncancerdrmurali.com/limb-sparing-surgery.html</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4862,7 +4884,7 @@
           <t>https://cioncancerdrmurali.com/osteosarcoma-limb-salvage.html</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4889,7 +4911,7 @@
           <t>https://cioncancerdrmurali.com/rectal-sphincter-preservation.html</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4916,7 +4938,7 @@
           <t>https://cioncancerdrmurali.com/low-anterior-resection.html</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4943,7 +4965,7 @@
           <t>https://cioncancerdrmurali.com/sigmoid-colon-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4970,7 +4992,7 @@
           <t>https://cioncancerdrmurali.com/laparoscopic-bowel-resection.html</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -4997,7 +5019,7 @@
           <t>https://cioncancerdrmurali.com/hemorrhoids-vs-rectal-cancer.html</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5024,7 +5046,7 @@
           <t>https://cioncancerdrmurali.com/liver-metastases-surgery.html</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5051,7 +5073,7 @@
           <t>https://cioncancerdrmurali.com/thermal-ablation-liver-tumours.html</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5078,7 +5100,7 @@
           <t>https://cioncancerdrmurali.com/bile-duct-repair-surgery.html</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5105,7 +5127,7 @@
           <t>https://cioncancerdrmurali.com/cholecystectomy-gallbladder-cancer.html</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5132,7 +5154,7 @@
           <t>https://cioncancerdrmurali.com/total-gastrectomy-recovery.html</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5159,7 +5181,7 @@
           <t>https://cioncancerdrmurali.com/small-bowel-resection.html</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5186,7 +5208,7 @@
           <t>https://cioncancerdrmurali.com/peritoneal-wash-cytology.html</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5213,7 +5235,7 @@
           <t>https://cioncancerdrmurali.com/second-look-surgery-ovarian.html</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5240,7 +5262,7 @@
           <t>https://cioncancerdrmurali.com/interval-debulking-surgery.html</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5267,7 +5289,7 @@
           <t>https://cioncancerdrmurali.com/cancer-surgery-diabetes.html</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5294,7 +5316,7 @@
           <t>https://cioncancerdrmurali.com/anastomosis-leak-prevention.html</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5321,7 +5343,7 @@
           <t>https://cioncancerdrmurali.com/ewing-sarcoma-treatment.html</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5348,7 +5370,7 @@
           <t>https://cioncancerdrmurali.com/synovial-sarcoma-treatment.html</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5375,7 +5397,7 @@
           <t>https://cioncancerdrmurali.com/amputation-bone-cancer.html</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5402,7 +5424,7 @@
           <t>https://cioncancerdrmurali.com/right-hemicolectomy.html</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5429,7 +5451,7 @@
           <t>https://cioncancerdrmurali.com/left-hemicolectomy.html</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5456,7 +5478,7 @@
           <t>https://cioncancerdrmurali.com/d2-lymphadenectomy-gastric.html</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5483,7 +5505,7 @@
           <t>https://cioncancerdrmurali.com/portal-vein-embolization.html</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5510,7 +5532,7 @@
           <t>https://cioncancerdrmurali.com/distal-pancreatectomy.html</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5537,7 +5559,7 @@
           <t>https://cioncancerdrmurali.com/radical-cholecystectomy-gallbladder.html</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5564,7 +5586,7 @@
           <t>https://cioncancerdrmurali.com/gist-tumour-treatment.html</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5591,7 +5613,7 @@
           <t>https://cioncancerdrmurali.com/mesenteric-tumour-resection.html</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5618,7 +5640,7 @@
           <t>https://cioncancerdrmurali.com/colon-cancer-peritoneal-spread.html</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5645,7 +5667,7 @@
           <t>https://cioncancerdrmurali.com/uterine-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5672,7 +5694,7 @@
           <t>https://cioncancerdrmurali.com/malignant-ascites-management.html</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5699,7 +5721,7 @@
           <t>https://cioncancerdrmurali.com/laparoscopic-staging-peritoneal.html</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5726,7 +5748,7 @@
           <t>https://cioncancerdrmurali.com/transverse-colon-cancer.html</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5753,7 +5775,7 @@
           <t>https://cioncancerdrmurali.com/anorectal-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5780,7 +5802,7 @@
           <t>https://cioncancerdrmurali.com/diverticulitis-vs-colon-cancer.html</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5807,7 +5829,7 @@
           <t>https://cioncancerdrmurali.com/phantom-limb-pain-management.html</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5834,7 +5856,7 @@
           <t>https://cioncancerdrmurali.com/intraoperative-bleeding-management.html</t>
         </is>
       </c>
-      <c r="E46" s="12" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5861,7 +5883,7 @@
           <t>https://cioncancerdrmurali.com/microwave-ablation-liver.html</t>
         </is>
       </c>
-      <c r="E47" s="11" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5888,7 +5910,7 @@
           <t>https://cioncancerdrmurali.com/proximal-gastrectomy.html</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5915,7 +5937,7 @@
           <t>https://cioncancerdrmurali.com/pancreatic-resection-recovery.html</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5942,7 +5964,7 @@
           <t>https://cioncancerdrmurali.com/abdominoperineal-resection.html</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5969,7 +5991,7 @@
           <t>https://cioncancerdrmurali.com/stoma-reversal-surgery.html</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -5996,7 +6018,7 @@
           <t>https://cioncancerdrmurali.com/eras-protocol-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E52" s="12" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -6023,7 +6045,7 @@
           <t>https://cioncancerdrmurali.com/cancer-surgery-blood-loss.html</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E53" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -6728,29 +6750,29 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Oral cancer surgery treatment</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>oral-cancer-surgery</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>https://cioncancerdrsandeep.com/oral-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Today →</t>
         </is>
       </c>
     </row>
@@ -6775,7 +6797,7 @@
           <t>https://cioncancerdrsandeep.com/tongue-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -6802,7 +6824,7 @@
           <t>https://cioncancerdrsandeep.com/lip-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -6829,7 +6851,7 @@
           <t>https://cioncancerdrsandeep.com/buccal-mucosa-cancer.html</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -6856,7 +6878,7 @@
           <t>https://cioncancerdrsandeep.com/floor-of-mouth-cancer.html</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -6883,7 +6905,7 @@
           <t>https://cioncancerdrsandeep.com/laryngeal-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -6910,7 +6932,7 @@
           <t>https://cioncancerdrsandeep.com/laryngectomy-voice-rehab.html</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -6937,7 +6959,7 @@
           <t>https://cioncancerdrsandeep.com/hypopharyngeal-cancer.html</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -6964,7 +6986,7 @@
           <t>https://cioncancerdrsandeep.com/oropharyngeal-cancer-hpv.html</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -6991,7 +7013,7 @@
           <t>https://cioncancerdrsandeep.com/tonsil-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7018,7 +7040,7 @@
           <t>https://cioncancerdrsandeep.com/nasopharyngeal-cancer.html</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7045,7 +7067,7 @@
           <t>https://cioncancerdrsandeep.com/nasal-cavity-cancer.html</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7072,7 +7094,7 @@
           <t>https://cioncancerdrsandeep.com/salivary-gland-cancer.html</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7099,7 +7121,7 @@
           <t>https://cioncancerdrsandeep.com/parotid-gland-surgery.html</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7126,7 +7148,7 @@
           <t>https://cioncancerdrsandeep.com/neck-dissection-types.html</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7153,7 +7175,7 @@
           <t>https://cioncancerdrsandeep.com/modified-radical-neck-dissection.html</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7180,7 +7202,7 @@
           <t>https://cioncancerdrsandeep.com/total-thyroidectomy.html</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7207,7 +7229,7 @@
           <t>https://cioncancerdrsandeep.com/papillary-thyroid-cancer.html</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7234,7 +7256,7 @@
           <t>https://cioncancerdrsandeep.com/follicular-thyroid-cancer.html</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7261,7 +7283,7 @@
           <t>https://cioncancerdrsandeep.com/medullary-thyroid-cancer.html</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7288,7 +7310,7 @@
           <t>https://cioncancerdrsandeep.com/thyroid-cancer-recurrence.html</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7315,7 +7337,7 @@
           <t>https://cioncancerdrsandeep.com/skull-base-tumour-surgery.html</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7342,7 +7364,7 @@
           <t>https://cioncancerdrsandeep.com/paraganglioma-treatment.html</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7369,7 +7391,7 @@
           <t>https://cioncancerdrsandeep.com/adenoid-cystic-carcinoma.html</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7396,7 +7418,7 @@
           <t>https://cioncancerdrsandeep.com/mucoepidermoid-carcinoma.html</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7423,7 +7445,7 @@
           <t>https://cioncancerdrsandeep.com/head-neck-cancer-trismus.html</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7450,7 +7472,7 @@
           <t>https://cioncancerdrsandeep.com/xerostomia-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7477,7 +7499,7 @@
           <t>https://cioncancerdrsandeep.com/dysphagia-head-neck-cancer.html</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7504,7 +7526,7 @@
           <t>https://cioncancerdrsandeep.com/head-neck-cancer-rehabilitation.html</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7531,7 +7553,7 @@
           <t>https://cioncancerdrsandeep.com/speech-therapy-laryngectomy.html</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7558,7 +7580,7 @@
           <t>https://cioncancerdrsandeep.com/neck-lump-causes.html</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7585,7 +7607,7 @@
           <t>https://cioncancerdrsandeep.com/hoarseness-cancer-signs.html</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7612,7 +7634,7 @@
           <t>https://cioncancerdrsandeep.com/mouth-ulcer-cancer-warning.html</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7639,7 +7661,7 @@
           <t>https://cioncancerdrsandeep.com/leukoplakia-oral-cancer.html</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7666,7 +7688,7 @@
           <t>https://cioncancerdrsandeep.com/submucous-fibrosis-cancer.html</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7693,7 +7715,7 @@
           <t>https://cioncancerdrsandeep.com/tobacco-oral-cancer.html</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7720,7 +7742,7 @@
           <t>https://cioncancerdrsandeep.com/base-of-tongue-cancer.html</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7747,7 +7769,7 @@
           <t>https://cioncancerdrsandeep.com/partial-laryngectomy.html</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7774,7 +7796,7 @@
           <t>https://cioncancerdrsandeep.com/palate-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7801,7 +7823,7 @@
           <t>https://cioncancerdrsandeep.com/jaw-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7828,7 +7850,7 @@
           <t>https://cioncancerdrsandeep.com/paranasal-sinus-cancer.html</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7855,7 +7877,7 @@
           <t>https://cioncancerdrsandeep.com/anaplastic-thyroid-cancer.html</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7882,7 +7904,7 @@
           <t>https://cioncancerdrsandeep.com/head-neck-cancer-hyderabad.html</t>
         </is>
       </c>
-      <c r="E46" s="12" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7909,7 +7931,7 @@
           <t>https://cioncancerdrsandeep.com/swallowing-therapy-cancer.html</t>
         </is>
       </c>
-      <c r="E47" s="11" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7936,7 +7958,7 @@
           <t>https://cioncancerdrsandeep.com/radiation-head-neck-surgery.html</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7963,7 +7985,7 @@
           <t>https://cioncancerdrsandeep.com/chemotherapy-head-neck-cancer.html</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -7990,7 +8012,7 @@
           <t>https://cioncancerdrsandeep.com/head-neck-cancer-nutrition.html</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -8017,7 +8039,7 @@
           <t>https://cioncancerdrsandeep.com/tracheostomy-care-cancer.html</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -8044,7 +8066,7 @@
           <t>https://cioncancerdrsandeep.com/reconstruction-head-neck-cancer.html</t>
         </is>
       </c>
-      <c r="E52" s="12" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -8071,7 +8093,7 @@
           <t>https://cioncancerdrsandeep.com/head-neck-cancer-surgeon-questions.html</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E53" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -8776,29 +8798,29 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Understanding cancer immunotherapy</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>understanding-immunotherapy</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>https://cioncancerdrkiranmayee.com/understanding-immunotherapy.html</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Today →</t>
         </is>
       </c>
     </row>
@@ -8823,7 +8845,7 @@
           <t>https://cioncancerdrkiranmayee.com/lung-cancer-types-stages.html</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -8850,7 +8872,7 @@
           <t>https://cioncancerdrkiranmayee.com/hormone-receptor-breast-cancer.html</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -8877,7 +8899,7 @@
           <t>https://cioncancerdrkiranmayee.com/non-hodgkin-lymphoma.html</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -8904,7 +8926,7 @@
           <t>https://cioncancerdrkiranmayee.com/chronic-myeloid-leukemia.html</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -8931,7 +8953,7 @@
           <t>https://cioncancerdrkiranmayee.com/melanoma-treatment.html</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -8958,7 +8980,7 @@
           <t>https://cioncancerdrkiranmayee.com/pancreatic-cancer-signs.html</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -8985,7 +9007,7 @@
           <t>https://cioncancerdrkiranmayee.com/liver-cancer-treatment-hyderabad.html</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9012,7 +9034,7 @@
           <t>https://cioncancerdrkiranmayee.com/uterine-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9039,7 +9061,7 @@
           <t>https://cioncancerdrkiranmayee.com/bone-cancer-types.html</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9066,7 +9088,7 @@
           <t>https://cioncancerdrkiranmayee.com/soft-tissue-sarcoma.html</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9093,7 +9115,7 @@
           <t>https://cioncancerdrkiranmayee.com/neuroendocrine-tumours.html</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9120,7 +9142,7 @@
           <t>https://cioncancerdrkiranmayee.com/bile-duct-cancer.html</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9147,7 +9169,7 @@
           <t>https://cioncancerdrkiranmayee.com/cancer-blood-clots-dvt.html</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9174,7 +9196,7 @@
           <t>https://cioncancerdrkiranmayee.com/checkpoint-inhibitors-immunotherapy.html</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9201,7 +9223,7 @@
           <t>https://cioncancerdrkiranmayee.com/car-t-cell-therapy.html</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9228,7 +9250,7 @@
           <t>https://cioncancerdrkiranmayee.com/parp-inhibitors-cancer.html</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9255,7 +9277,7 @@
           <t>https://cioncancerdrkiranmayee.com/cdk-inhibitors-breast-cancer.html</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9282,7 +9304,7 @@
           <t>https://cioncancerdrkiranmayee.com/combination-chemotherapy.html</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9309,7 +9331,7 @@
           <t>https://cioncancerdrkiranmayee.com/weight-management-chemotherapy.html</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9336,7 +9358,7 @@
           <t>https://cioncancerdrkiranmayee.com/cancer-mental-health.html</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9363,7 +9385,7 @@
           <t>https://cioncancerdrkiranmayee.com/exercise-during-cancer.html</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9390,7 +9412,7 @@
           <t>https://cioncancerdrkiranmayee.com/cancer-pain-types.html</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9417,7 +9439,7 @@
           <t>https://cioncancerdrkiranmayee.com/cancer-end-of-life-care.html</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9444,7 +9466,7 @@
           <t>https://cioncancerdrkiranmayee.com/cancer-rehabilitation.html</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9471,7 +9493,7 @@
           <t>https://cioncancerdrkiranmayee.com/return-to-work-cancer.html</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9498,7 +9520,7 @@
           <t>https://cioncancerdrkiranmayee.com/cancer-insurance-india.html</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9525,7 +9547,7 @@
           <t>https://cioncancerdrkiranmayee.com/government-cancer-schemes-india.html</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9552,7 +9574,7 @@
           <t>https://cioncancerdrkiranmayee.com/telemedicine-cancer-followup.html</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9579,7 +9601,7 @@
           <t>https://cioncancerdrkiranmayee.com/cancer-young-adults.html</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9606,7 +9628,7 @@
           <t>https://cioncancerdrkiranmayee.com/antibody-drug-conjugates.html</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9633,7 +9655,7 @@
           <t>https://cioncancerdrkiranmayee.com/maintenance-therapy-cancer.html</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9660,7 +9682,7 @@
           <t>https://cioncancerdrkiranmayee.com/adjuvant-neoadjuvant-therapy.html</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9687,7 +9709,7 @@
           <t>https://cioncancerdrkiranmayee.com/dose-dense-chemotherapy.html</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9714,7 +9736,7 @@
           <t>https://cioncancerdrkiranmayee.com/growth-factors-chemotherapy.html</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9741,7 +9763,7 @@
           <t>https://cioncancerdrkiranmayee.com/febrile-neutropenia.html</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9768,7 +9790,7 @@
           <t>https://cioncancerdrkiranmayee.com/cardio-oncology-cancer.html</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9795,7 +9817,7 @@
           <t>https://cioncancerdrkiranmayee.com/second-primary-cancer.html</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9822,7 +9844,7 @@
           <t>https://cioncancerdrkiranmayee.com/cancer-treatment-at-home.html</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9849,7 +9871,7 @@
           <t>https://cioncancerdrkiranmayee.com/oral-cancer-prevention.html</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9876,7 +9898,7 @@
           <t>https://cioncancerdrkiranmayee.com/colon-cancer-prevention.html</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9903,7 +9925,7 @@
           <t>https://cioncancerdrkiranmayee.com/pancreatic-cancer-warning-signs.html</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9930,7 +9952,7 @@
           <t>https://cioncancerdrkiranmayee.com/vulvar-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E46" s="12" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9957,7 +9979,7 @@
           <t>https://cioncancerdrkiranmayee.com/penile-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E47" s="11" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -9984,7 +10006,7 @@
           <t>https://cioncancerdrkiranmayee.com/anal-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -10011,7 +10033,7 @@
           <t>https://cioncancerdrkiranmayee.com/adrenal-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -10038,7 +10060,7 @@
           <t>https://cioncancerdrkiranmayee.com/cancer-genetic-counselling.html</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -10065,7 +10087,7 @@
           <t>https://cioncancerdrkiranmayee.com/complementary-medicine-cancer.html</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -10092,7 +10114,7 @@
           <t>https://cioncancerdrkiranmayee.com/hospice-care-cancer.html</t>
         </is>
       </c>
-      <c r="E52" s="12" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -10119,7 +10141,7 @@
           <t>https://cioncancerdrkiranmayee.com/cancer-caregiver-burnout.html</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E53" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -10824,29 +10846,29 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Bone marrow transplant explained</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>bone-marrow-transplant-explained</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>https://cioncancerdrbasudev.com/bone-marrow-transplant-explained.html</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Today →</t>
         </is>
       </c>
     </row>
@@ -10871,7 +10893,7 @@
           <t>https://cioncancerdrbasudev.com/autologous-bmt.html</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -10898,7 +10920,7 @@
           <t>https://cioncancerdrbasudev.com/allogeneic-bmt.html</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -10925,7 +10947,7 @@
           <t>https://cioncancerdrbasudev.com/stem-cell-donation.html</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -10952,7 +10974,7 @@
           <t>https://cioncancerdrbasudev.com/bone-marrow-donor-compatibility.html</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -10979,7 +11001,7 @@
           <t>https://cioncancerdrbasudev.com/bmt-recovery-timeline.html</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11006,7 +11028,7 @@
           <t>https://cioncancerdrbasudev.com/graft-versus-host-disease.html</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11033,7 +11055,7 @@
           <t>https://cioncancerdrbasudev.com/chronic-gvhd-management.html</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11060,7 +11082,7 @@
           <t>https://cioncancerdrbasudev.com/what-is-leukemia.html</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11087,7 +11109,7 @@
           <t>https://cioncancerdrbasudev.com/acute-myeloid-leukemia.html</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11114,7 +11136,7 @@
           <t>https://cioncancerdrbasudev.com/acute-lymphoblastic-leukemia.html</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11141,7 +11163,7 @@
           <t>https://cioncancerdrbasudev.com/chronic-lymphocytic-leukemia.html</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11168,7 +11190,7 @@
           <t>https://cioncancerdrbasudev.com/hairy-cell-leukemia.html</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11195,7 +11217,7 @@
           <t>https://cioncancerdrbasudev.com/myelodysplastic-syndrome.html</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11222,7 +11244,7 @@
           <t>https://cioncancerdrbasudev.com/myelofibrosis-treatment.html</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11249,7 +11271,7 @@
           <t>https://cioncancerdrbasudev.com/polycythemia-vera.html</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11276,7 +11298,7 @@
           <t>https://cioncancerdrbasudev.com/essential-thrombocythemia.html</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11303,7 +11325,7 @@
           <t>https://cioncancerdrbasudev.com/aplastic-anemia-treatment.html</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11330,7 +11352,7 @@
           <t>https://cioncancerdrbasudev.com/thalassemia-stem-cell-therapy.html</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11357,7 +11379,7 @@
           <t>https://cioncancerdrbasudev.com/hodgkin-lymphoma-treatment.html</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11384,7 +11406,7 @@
           <t>https://cioncancerdrbasudev.com/diffuse-large-b-cell-lymphoma.html</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11411,7 +11433,7 @@
           <t>https://cioncancerdrbasudev.com/follicular-lymphoma.html</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11438,7 +11460,7 @@
           <t>https://cioncancerdrbasudev.com/mantle-cell-lymphoma.html</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11465,7 +11487,7 @@
           <t>https://cioncancerdrbasudev.com/burkitt-lymphoma.html</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11492,7 +11514,7 @@
           <t>https://cioncancerdrbasudev.com/t-cell-lymphoma.html</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11519,7 +11541,7 @@
           <t>https://cioncancerdrbasudev.com/waldenstrom-macroglobulinemia.html</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11546,7 +11568,7 @@
           <t>https://cioncancerdrbasudev.com/multiple-myeloma-bone-pain.html</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11573,7 +11595,7 @@
           <t>https://cioncancerdrbasudev.com/smoldering-myeloma.html</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11600,7 +11622,7 @@
           <t>https://cioncancerdrbasudev.com/bortezomib-myeloma.html</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11627,7 +11649,7 @@
           <t>https://cioncancerdrbasudev.com/daratumumab-myeloma.html</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11654,7 +11676,7 @@
           <t>https://cioncancerdrbasudev.com/venetoclax-blood-cancer.html</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11681,7 +11703,7 @@
           <t>https://cioncancerdrbasudev.com/ibrutinib-cll.html</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11708,7 +11730,7 @@
           <t>https://cioncancerdrbasudev.com/rituximab-lymphoma.html</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11735,7 +11757,7 @@
           <t>https://cioncancerdrbasudev.com/bone-marrow-biopsy-procedure.html</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11762,7 +11784,7 @@
           <t>https://cioncancerdrbasudev.com/cbc-cancer-interpretation.html</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11789,7 +11811,7 @@
           <t>https://cioncancerdrbasudev.com/flow-cytometry-cancer.html</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11816,7 +11838,7 @@
           <t>https://cioncancerdrbasudev.com/fish-testing-blood-cancer.html</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11843,7 +11865,7 @@
           <t>https://cioncancerdrbasudev.com/blood-cancer-treatment-hyderabad.html</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11870,7 +11892,7 @@
           <t>https://cioncancerdrbasudev.com/bmt-cost-india.html</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11897,7 +11919,7 @@
           <t>https://cioncancerdrbasudev.com/life-after-bmt.html</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11924,7 +11946,7 @@
           <t>https://cioncancerdrbasudev.com/infections-after-bmt.html</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11951,7 +11973,7 @@
           <t>https://cioncancerdrbasudev.com/engraftment-syndrome.html</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -11978,7 +12000,7 @@
           <t>https://cioncancerdrbasudev.com/peripheral-blood-stem-cell-harvest.html</t>
         </is>
       </c>
-      <c r="E46" s="12" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -12005,7 +12027,7 @@
           <t>https://cioncancerdrbasudev.com/cord-blood-transplant.html</t>
         </is>
       </c>
-      <c r="E47" s="11" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -12032,7 +12054,7 @@
           <t>https://cioncancerdrbasudev.com/haploidentical-transplant.html</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -12059,7 +12081,7 @@
           <t>https://cioncancerdrbasudev.com/reduced-intensity-conditioning-bmt.html</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -12086,7 +12108,7 @@
           <t>https://cioncancerdrbasudev.com/nk-cell-lymphoma.html</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -12113,7 +12135,7 @@
           <t>https://cioncancerdrbasudev.com/amyloidosis-blood-cancer.html</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -12140,7 +12162,7 @@
           <t>https://cioncancerdrbasudev.com/bone-marrow-failure-syndromes.html</t>
         </is>
       </c>
-      <c r="E52" s="12" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -12167,7 +12189,7 @@
           <t>https://cioncancerdrbasudev.com/blood-cancer-diet-nutrition.html</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E53" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -12872,29 +12894,29 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>What is radiation therapy</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>what-is-radiation-therapy</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>https://cioncancerdrraghvendra.com/what-is-radiation-therapy.html</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Today →</t>
         </is>
       </c>
     </row>
@@ -12919,7 +12941,7 @@
           <t>https://cioncancerdrraghvendra.com/external-beam-radiation.html</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -12946,7 +12968,7 @@
           <t>https://cioncancerdrraghvendra.com/imrt-radiation-therapy.html</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -12973,7 +12995,7 @@
           <t>https://cioncancerdrraghvendra.com/igrt-radiation-therapy.html</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13000,7 +13022,7 @@
           <t>https://cioncancerdrraghvendra.com/stereotactic-radiosurgery.html</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13027,7 +13049,7 @@
           <t>https://cioncancerdrraghvendra.com/sbrt-radiation-therapy.html</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13054,7 +13076,7 @@
           <t>https://cioncancerdrraghvendra.com/brachytherapy-explained.html</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13081,7 +13103,7 @@
           <t>https://cioncancerdrraghvendra.com/high-dose-rate-brachytherapy.html</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13108,7 +13130,7 @@
           <t>https://cioncancerdrraghvendra.com/breast-cancer-radiation.html</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13135,7 +13157,7 @@
           <t>https://cioncancerdrraghvendra.com/cervical-cancer-radiation.html</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13162,7 +13184,7 @@
           <t>https://cioncancerdrraghvendra.com/prostate-cancer-radiation.html</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13189,7 +13211,7 @@
           <t>https://cioncancerdrraghvendra.com/lung-cancer-radiation.html</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13216,7 +13238,7 @@
           <t>https://cioncancerdrraghvendra.com/head-neck-radiation-therapy.html</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13243,7 +13265,7 @@
           <t>https://cioncancerdrraghvendra.com/rectal-cancer-radiation.html</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13270,7 +13292,7 @@
           <t>https://cioncancerdrraghvendra.com/whole-brain-radiation.html</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13297,7 +13319,7 @@
           <t>https://cioncancerdrraghvendra.com/palliative-radiation-bone-pain.html</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13324,7 +13346,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-therapy-side-effects.html</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13351,7 +13373,7 @@
           <t>https://cioncancerdrraghvendra.com/skin-reactions-radiation.html</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13378,7 +13400,7 @@
           <t>https://cioncancerdrraghvendra.com/fatigue-radiation-therapy.html</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13405,7 +13427,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-mucositis.html</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13432,7 +13454,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-enteritis.html</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13459,7 +13481,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-cystitis.html</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13486,7 +13508,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-therapy-simulation.html</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13513,7 +13535,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-treatment-planning.html</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13540,7 +13562,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-therapy-fractions.html</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13567,7 +13589,7 @@
           <t>https://cioncancerdrraghvendra.com/hypofractionated-radiation.html</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13594,7 +13616,7 @@
           <t>https://cioncancerdrraghvendra.com/concurrent-chemoradiation.html</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13621,7 +13643,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-brain-metastases.html</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13648,7 +13670,7 @@
           <t>https://cioncancerdrraghvendra.com/spinal-cord-compression-radiation.html</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13675,7 +13697,7 @@
           <t>https://cioncancerdrraghvendra.com/sabr-liver-tumours.html</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13702,7 +13724,7 @@
           <t>https://cioncancerdrraghvendra.com/radioiodine-therapy-thyroid.html</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13729,7 +13751,7 @@
           <t>https://cioncancerdrraghvendra.com/prrt-neuroendocrine-tumours.html</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13756,7 +13778,7 @@
           <t>https://cioncancerdrraghvendra.com/lutetium-dotatate-therapy.html</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13783,7 +13805,7 @@
           <t>https://cioncancerdrraghvendra.com/y90-radioembolization.html</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13810,7 +13832,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-vs-surgery.html</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13837,7 +13859,7 @@
           <t>https://cioncancerdrraghvendra.com/proton-therapy-vs-radiation.html</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13864,7 +13886,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-quality-of-life.html</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13891,7 +13913,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-therapy-myths.html</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13918,7 +13940,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-therapy-cost-hyderabad.html</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13945,7 +13967,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-therapy-safety.html</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13972,7 +13994,7 @@
           <t>https://cioncancerdrraghvendra.com/re-irradiation-cancer.html</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -13999,7 +14021,7 @@
           <t>https://cioncancerdrraghvendra.com/second-cancer-after-radiation.html</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -14026,7 +14048,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-protection-family.html</t>
         </is>
       </c>
-      <c r="E46" s="12" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -14053,7 +14075,7 @@
           <t>https://cioncancerdrraghvendra.com/radiation-therapy-fertility.html</t>
         </is>
       </c>
-      <c r="E47" s="11" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -14080,7 +14102,7 @@
           <t>https://cioncancerdrraghvendra.com/accelerated-partial-breast-irradiation.html</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -14107,7 +14129,7 @@
           <t>https://cioncancerdrraghvendra.com/intraoperative-radiation-therapy.html</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -14134,7 +14156,7 @@
           <t>https://cioncancerdrraghvendra.com/total-body-irradiation.html</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -14161,7 +14183,7 @@
           <t>https://cioncancerdrraghvendra.com/radiofrequency-ablation-cancer.html</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -14188,7 +14210,7 @@
           <t>https://cioncancerdrraghvendra.com/tace-liver-cancer.html</t>
         </is>
       </c>
-      <c r="E52" s="12" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -14215,7 +14237,7 @@
           <t>https://cioncancerdrraghvendra.com/esophageal-cancer-radiation.html</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E53" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -14920,29 +14942,29 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Colon cancer treatment options</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>colon-cancer-treatment</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>https://cioncancerdrcraghavendra.info/colon-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Today →</t>
         </is>
       </c>
     </row>
@@ -14967,7 +14989,7 @@
           <t>https://cioncancerdrcraghavendra.info/rectal-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -14994,7 +15016,7 @@
           <t>https://cioncancerdrcraghavendra.info/appendix-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15021,7 +15043,7 @@
           <t>https://cioncancerdrcraghavendra.info/peritoneal-carcinomatosis.html</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15048,7 +15070,7 @@
           <t>https://cioncancerdrcraghavendra.info/cea-tumor-marker.html</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15075,7 +15097,7 @@
           <t>https://cioncancerdrcraghavendra.info/ca125-test-explained.html</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15102,7 +15124,7 @@
           <t>https://cioncancerdrcraghavendra.info/ca19-9-test-explained.html</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15129,7 +15151,7 @@
           <t>https://cioncancerdrcraghavendra.info/afp-test-liver-cancer.html</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15156,7 +15178,7 @@
           <t>https://cioncancerdrcraghavendra.info/psa-test-explained.html</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15183,7 +15205,7 @@
           <t>https://cioncancerdrcraghavendra.info/core-needle-biopsy.html</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15210,7 +15232,7 @@
           <t>https://cioncancerdrcraghavendra.info/liquid-biopsy-cancer.html</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15237,7 +15259,7 @@
           <t>https://cioncancerdrcraghavendra.info/next-generation-sequencing-cancer.html</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15264,7 +15286,7 @@
           <t>https://cioncancerdrcraghavendra.info/microsatellite-instability.html</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15291,7 +15313,7 @@
           <t>https://cioncancerdrcraghavendra.info/kras-mutation-colorectal.html</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15318,7 +15340,7 @@
           <t>https://cioncancerdrcraghavendra.info/egfr-mutation-lung-cancer.html</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15345,7 +15367,7 @@
           <t>https://cioncancerdrcraghavendra.info/braf-mutation-cancer.html</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15372,7 +15394,7 @@
           <t>https://cioncancerdrcraghavendra.info/pdl1-expression-cancer.html</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15399,7 +15421,7 @@
           <t>https://cioncancerdrcraghavendra.info/precision-oncology-hyderabad.html</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15426,7 +15448,7 @@
           <t>https://cioncancerdrcraghavendra.info/cancer-diet-myths.html</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15453,7 +15475,7 @@
           <t>https://cioncancerdrcraghavendra.info/sugar-cancer-link.html</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15480,7 +15502,7 @@
           <t>https://cioncancerdrcraghavendra.info/alcohol-cancer-risk.html</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15507,7 +15529,7 @@
           <t>https://cioncancerdrcraghavendra.info/obesity-cancer-risk.html</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15534,7 +15556,7 @@
           <t>https://cioncancerdrcraghavendra.info/cancer-prevention-strategies.html</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15561,7 +15583,7 @@
           <t>https://cioncancerdrcraghavendra.info/cancer-early-detection-india.html</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15588,7 +15610,7 @@
           <t>https://cioncancerdrcraghavendra.info/colonoscopy-screening.html</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15615,7 +15637,7 @@
           <t>https://cioncancerdrcraghavendra.info/mammography-screening.html</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15642,7 +15664,7 @@
           <t>https://cioncancerdrcraghavendra.info/pap-smear-screening.html</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15669,7 +15691,7 @@
           <t>https://cioncancerdrcraghavendra.info/recist-criteria-cancer.html</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15696,7 +15718,7 @@
           <t>https://cioncancerdrcraghavendra.info/adjuvant-chemotherapy-explained.html</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15723,7 +15745,7 @@
           <t>https://cioncancerdrcraghavendra.info/bone-marrow-suppression.html</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15750,7 +15772,7 @@
           <t>https://cioncancerdrcraghavendra.info/cancer-biomarkers-explained.html</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15777,7 +15799,7 @@
           <t>https://cioncancerdrcraghavendra.info/biliary-tract-cancer.html</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15804,7 +15826,7 @@
           <t>https://cioncancerdrcraghavendra.info/duodenal-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15831,7 +15853,7 @@
           <t>https://cioncancerdrcraghavendra.info/small-intestine-cancer-treatment.html</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15858,7 +15880,7 @@
           <t>https://cioncancerdrcraghavendra.info/tumor-biopsy-types.html</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15885,7 +15907,7 @@
           <t>https://cioncancerdrcraghavendra.info/smoking-cancer-prevention.html</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15912,7 +15934,7 @@
           <t>https://cioncancerdrcraghavendra.info/red-meat-cancer-risk.html</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15939,7 +15961,7 @@
           <t>https://cioncancerdrcraghavendra.info/stress-cancer-link.html</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15966,7 +15988,7 @@
           <t>https://cioncancerdrcraghavendra.info/turmeric-cancer-research.html</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -15993,7 +16015,7 @@
           <t>https://cioncancerdrcraghavendra.info/cancer-treatment-cost-india.html</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -16020,7 +16042,7 @@
           <t>https://cioncancerdrcraghavendra.info/ayushman-bharat-cancer.html</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -16047,7 +16069,7 @@
           <t>https://cioncancerdrcraghavendra.info/cancer-screening-age-guidelines.html</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -16074,7 +16096,7 @@
           <t>https://cioncancerdrcraghavendra.info/tumor-mutational-burden.html</t>
         </is>
       </c>
-      <c r="E46" s="12" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -16101,7 +16123,7 @@
           <t>https://cioncancerdrcraghavendra.info/msi-high-immunotherapy.html</t>
         </is>
       </c>
-      <c r="E47" s="11" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -16128,7 +16150,7 @@
           <t>https://cioncancerdrcraghavendra.info/colorectal-cancer-followup.html</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -16155,7 +16177,7 @@
           <t>https://cioncancerdrcraghavendra.info/kras-wildtype-colorectal.html</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -16182,7 +16204,7 @@
           <t>https://cioncancerdrcraghavendra.info/stoma-care-colorectal.html</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -16209,7 +16231,7 @@
           <t>https://cioncancerdrcraghavendra.info/rectal-bleeding-cancer-signs.html</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -16236,7 +16258,7 @@
           <t>https://cioncancerdrcraghavendra.info/bowel-habits-cancer-signs.html</t>
         </is>
       </c>
-      <c r="E52" s="12" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -16263,7 +16285,7 @@
           <t>https://cioncancerdrcraghavendra.info/iron-deficiency-anaemia-cancer.html</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E53" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -16996,29 +17018,29 @@
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>What is HIPEC surgery</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>what-is-hipec</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>https://cioncancerdrimad.com/what-is-hipec.html</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
+      <c r="E4" s="16" t="inlineStr">
+        <is>
+          <t>Today →</t>
         </is>
       </c>
     </row>
@@ -17043,7 +17065,7 @@
           <t>https://cioncancerdrimad.com/hipec-ovarian-cancer.html</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17070,7 +17092,7 @@
           <t>https://cioncancerdrimad.com/hipec-colorectal-cancer.html</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17097,7 +17119,7 @@
           <t>https://cioncancerdrimad.com/hipec-gastric-cancer.html</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17124,7 +17146,7 @@
           <t>https://cioncancerdrimad.com/pipac-procedure-explained.html</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17151,7 +17173,7 @@
           <t>https://cioncancerdrimad.com/pipac-vs-hipec.html</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17178,7 +17200,7 @@
           <t>https://cioncancerdrimad.com/cytoreductive-surgery-explained.html</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17205,7 +17227,7 @@
           <t>https://cioncancerdrimad.com/pci-score-peritoneal-cancer.html</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17232,7 +17254,7 @@
           <t>https://cioncancerdrimad.com/peritoneal-metastases-treatment.html</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17259,7 +17281,7 @@
           <t>https://cioncancerdrimad.com/pseudomyxoma-peritonei.html</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17286,7 +17308,7 @@
           <t>https://cioncancerdrimad.com/appendix-cancer-mucinous.html</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17313,7 +17335,7 @@
           <t>https://cioncancerdrimad.com/peritoneal-mesothelioma.html</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17340,7 +17362,7 @@
           <t>https://cioncancerdrimad.com/primary-peritoneal-cancer.html</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17367,7 +17389,7 @@
           <t>https://cioncancerdrimad.com/gastric-cancer-surgery-options.html</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17394,7 +17416,7 @@
           <t>https://cioncancerdrimad.com/total-gastrectomy-stomach-cancer.html</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17421,7 +17443,7 @@
           <t>https://cioncancerdrimad.com/d2-dissection-gastric-cancer.html</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17448,7 +17470,7 @@
           <t>https://cioncancerdrimad.com/esophagogastric-junction-cancer.html</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17475,7 +17497,7 @@
           <t>https://cioncancerdrimad.com/whipple-procedure-guide.html</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17502,7 +17524,7 @@
           <t>https://cioncancerdrimad.com/whipple-recovery-diet.html</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17529,7 +17551,7 @@
           <t>https://cioncancerdrimad.com/pylorus-preserving-whipple.html</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17556,7 +17578,7 @@
           <t>https://cioncancerdrimad.com/distal-pancreatectomy-splenectomy.html</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17583,7 +17605,7 @@
           <t>https://cioncancerdrimad.com/borderline-resectable-pancreatic.html</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17610,7 +17632,7 @@
           <t>https://cioncancerdrimad.com/hepatobiliary-cancer-hyderabad.html</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17637,7 +17659,7 @@
           <t>https://cioncancerdrimad.com/right-hepatectomy-liver-cancer.html</t>
         </is>
       </c>
-      <c r="E27" s="11" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17664,7 +17686,7 @@
           <t>https://cioncancerdrimad.com/klatskin-tumour-surgery.html</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17691,7 +17713,7 @@
           <t>https://cioncancerdrimad.com/gallbladder-cancer-surgery-options.html</t>
         </is>
       </c>
-      <c r="E29" s="11" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17718,7 +17740,7 @@
           <t>https://cioncancerdrimad.com/radical-cholecystectomy.html</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17745,7 +17767,7 @@
           <t>https://cioncancerdrimad.com/gist-treatment-imatinib.html</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E31" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17772,7 +17794,7 @@
           <t>https://cioncancerdrimad.com/retroperitoneal-tumour-surgery.html</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17799,7 +17821,7 @@
           <t>https://cioncancerdrimad.com/colorectal-liver-metastases-crs.html</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17826,7 +17848,7 @@
           <t>https://cioncancerdrimad.com/ovarian-cancer-hipec.html</t>
         </is>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17853,7 +17875,7 @@
           <t>https://cioncancerdrimad.com/brca-ovarian-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E35" s="11" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17880,7 +17902,7 @@
           <t>https://cioncancerdrimad.com/malignant-ascites-treatment.html</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17907,7 +17929,7 @@
           <t>https://cioncancerdrimad.com/laparoscopic-staging.html</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17934,7 +17956,7 @@
           <t>https://cioncancerdrimad.com/second-opinion-hipec.html</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17961,7 +17983,7 @@
           <t>https://cioncancerdrimad.com/hipec-cost-india.html</t>
         </is>
       </c>
-      <c r="E39" s="11" t="inlineStr">
+      <c r="E39" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -17988,7 +18010,7 @@
           <t>https://cioncancerdrimad.com/life-after-hipec.html</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18015,7 +18037,7 @@
           <t>https://cioncancerdrimad.com/recovery-cytoreductive-surgery.html</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
+      <c r="E41" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18042,7 +18064,7 @@
           <t>https://cioncancerdrimad.com/peritoneal-cancer-surgery-possible.html</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18069,7 +18091,7 @@
           <t>https://cioncancerdrimad.com/hipec-contraindications.html</t>
         </is>
       </c>
-      <c r="E43" s="11" t="inlineStr">
+      <c r="E43" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18096,7 +18118,7 @@
           <t>https://cioncancerdrimad.com/intraperitoneal-chemotherapy.html</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr">
+      <c r="E44" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18123,7 +18145,7 @@
           <t>https://cioncancerdrimad.com/gastric-cancer-peritoneal-spread.html</t>
         </is>
       </c>
-      <c r="E45" s="11" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18150,7 +18172,7 @@
           <t>https://cioncancerdrimad.com/appendix-rupture-cancer-risk.html</t>
         </is>
       </c>
-      <c r="E46" s="12" t="inlineStr">
+      <c r="E46" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18177,7 +18199,7 @@
           <t>https://cioncancerdrimad.com/liver-cancer-resection.html</t>
         </is>
       </c>
-      <c r="E47" s="11" t="inlineStr">
+      <c r="E47" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18204,7 +18226,7 @@
           <t>https://cioncancerdrimad.com/portal-vein-pancreatic-cancer.html</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18231,7 +18253,7 @@
           <t>https://cioncancerdrimad.com/gi-cancer-second-opinion-hyderabad.html</t>
         </is>
       </c>
-      <c r="E49" s="11" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18258,7 +18280,7 @@
           <t>https://cioncancerdrimad.com/peritoneal-cancer-survival.html</t>
         </is>
       </c>
-      <c r="E50" s="12" t="inlineStr">
+      <c r="E50" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18285,7 +18307,7 @@
           <t>https://cioncancerdrimad.com/laparoscopic-vs-open-cancer-surgery.html</t>
         </is>
       </c>
-      <c r="E51" s="11" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18312,7 +18334,7 @@
           <t>https://cioncancerdrimad.com/crs-hipec-vs-chemotherapy.html</t>
         </is>
       </c>
-      <c r="E52" s="12" t="inlineStr">
+      <c r="E52" s="11" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>
@@ -18339,7 +18361,7 @@
           <t>https://cioncancerdrimad.com/cancers-that-spread-to-peritoneum.html</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E53" s="12" t="inlineStr">
         <is>
           <t>Scheduled</t>
         </is>

</xml_diff>